<commit_message>
MR-12: spread the week calibration, build goldens through the contract
- calibration scales each target week to just under its figure, then closes the gap one
  unit at a time over the week's best sellers; no more negative line or one-day spike
- goldens are validated and dumped through NormalizedBatch
- regenerate deletes files it no longer produces, and --check flags them
- xlsx stored uncompressed so the bytes don't depend on the zlib build
- generated files are LF (xlsx binary) in .gitattributes
- 60_seed builds the manager's claims from its membership row
- build() returns its sales so render() generates once

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XfZQqYeq7SD8uXjzZBFDYG
</commit_message>
<xml_diff>
--- a/fixtures/sr/synthetic/productos_vendidos_L1_2026-10-11.xlsx
+++ b/fixtures/sr/synthetic/productos_vendidos_L1_2026-10-11.xlsx
@@ -496,19 +496,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E6" t="n">
         <v>65</v>
       </c>
       <c r="F6" t="n">
-        <v>3510</v>
+        <v>3640</v>
       </c>
       <c r="G6" t="n">
-        <v>9.75</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>3500.25</v>
+        <v>3640</v>
       </c>
     </row>
     <row r="7">
@@ -528,19 +528,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
         <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>2100</v>
+        <v>2250</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>2100</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="8">
@@ -560,19 +560,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E8" t="n">
         <v>70</v>
       </c>
       <c r="F8" t="n">
-        <v>2170</v>
+        <v>2310</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>2170</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="9">
@@ -592,19 +592,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" t="n">
         <v>75</v>
       </c>
       <c r="F9" t="n">
-        <v>1650</v>
+        <v>1725</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1650</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="10">
@@ -752,19 +752,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E14" t="n">
         <v>85</v>
       </c>
       <c r="F14" t="n">
-        <v>1615</v>
+        <v>1785</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1615</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="15">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E17" t="n">
         <v>45</v>
       </c>
       <c r="F17" t="n">
-        <v>990</v>
+        <v>1080</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>990</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="18">
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E29" t="n">
         <v>35</v>
       </c>
       <c r="F29" t="n">
-        <v>1120</v>
+        <v>1155</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1120</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="30">
@@ -1264,19 +1264,19 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E30" t="n">
         <v>35</v>
       </c>
       <c r="F30" t="n">
-        <v>735</v>
+        <v>770</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>735</v>
+        <v>770</v>
       </c>
     </row>
     <row r="31">
@@ -1328,19 +1328,19 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E32" t="n">
         <v>30</v>
       </c>
       <c r="F32" t="n">
-        <v>1590</v>
+        <v>1650</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1590</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="33">
@@ -1456,19 +1456,19 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>304</v>
+        <v>7</v>
       </c>
       <c r="E36" t="n">
         <v>25</v>
       </c>
       <c r="F36" t="n">
-        <v>7600</v>
+        <v>175</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>7600</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37">
@@ -1488,19 +1488,19 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E37" t="n">
         <v>45</v>
       </c>
       <c r="F37" t="n">
-        <v>990</v>
+        <v>1080</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>990</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="38">
@@ -1520,19 +1520,19 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E38" t="n">
         <v>45</v>
       </c>
       <c r="F38" t="n">
-        <v>360</v>
+        <v>405</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>360</v>
+        <v>405</v>
       </c>
     </row>
     <row r="39">
@@ -1552,19 +1552,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" t="n">
         <v>65</v>
       </c>
       <c r="F39" t="n">
-        <v>325</v>
+        <v>390</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>325</v>
+        <v>390</v>
       </c>
     </row>
     <row r="40">
@@ -1776,19 +1776,19 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E46" t="n">
         <v>15</v>
       </c>
       <c r="F46" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47">
@@ -1800,16 +1800,16 @@
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="n">
-        <v>842</v>
+        <v>565</v>
       </c>
       <c r="F47" t="n">
-        <v>37525</v>
+        <v>31200</v>
       </c>
       <c r="G47" t="n">
-        <v>9.75</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>37515.25</v>
+        <v>31200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MR-12: cancelled tickets with waiters, food cost figure, review fixes
- 17 cancelled tickets on Centro 2026-10-10 at ticket grain, every line voided by a waiter
  with a reason (13 H3 example 7); the day's cancellations come from them
- expected.json: cancellations by waiter and yesterday's food cost with its definition
- calibration leaves the Tuesday promo lines alone, so their discount stays exactly 15 %
- 60_seed: cancellation checks; membership check asserts the location, not a tautology
- 10_isolation: the postgres check counts only the test tenants' tickets

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XfZQqYeq7SD8uXjzZBFDYG
</commit_message>
<xml_diff>
--- a/fixtures/sr/synthetic/productos_vendidos_L1_2026-10-11.xlsx
+++ b/fixtures/sr/synthetic/productos_vendidos_L1_2026-10-11.xlsx
@@ -505,10 +505,10 @@
         <v>3640</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>3640</v>
+        <v>3635</v>
       </c>
     </row>
     <row r="7">
@@ -1806,10 +1806,10 @@
         <v>31200</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H47" t="n">
-        <v>31200</v>
+        <v>31195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>